<commit_message>
feat: Add Supabase + Vercel live deployment support
- Add Supabase sync engine (backend/supabase_sync.py) with watchlist, triggers, chart cache
- Add daily GitHub Actions workflow (.github/workflows/scan.yml) for 3:45 PM IST auto-scan
- Update backend/main.py to auto-push to Supabase after each pipeline run
- New frontend/index.html: dual-mode (Supabase cloud OR local FastAPI fallback)
  - Supabase JS v2 client with localStorage credential storage
  - Supabase config modal in header for easy connection by friend
  - SheetJS client-side Excel export (no backend required on Vercel)
  - Realtime Postgres LISTEN/NOTIFY for live trigger updates
  - Client-side chart fallback if backend unreachable
- Add supabase/schema.sql with RLS policies for public read access
- Add vercel.json routing config for static hosting
- Add .env.example, .gitignore, frontend/config.js
</commit_message>
<xml_diff>
--- a/Final_Trade_Triggers.xlsx
+++ b/Final_Trade_Triggers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,40 +548,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MAYURUNIQ</t>
+          <t>TARIL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mayur Uniquoters</t>
+          <t>T R I L</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="D2" t="n">
-        <v>24750</v>
+        <v>2320786</v>
       </c>
       <c r="E2" t="n">
-        <v>54000</v>
+        <v>6280999</v>
       </c>
       <c r="F2" t="n">
-        <v>2.18</v>
+        <v>2.71</v>
       </c>
       <c r="G2" t="n">
-        <v>179</v>
+        <v>304.1</v>
       </c>
       <c r="H2" t="n">
-        <v>208.5</v>
+        <v>391.5</v>
       </c>
       <c r="I2" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="J2" t="n">
-        <v>176.31</v>
+        <v>371.3</v>
       </c>
       <c r="K2" t="n">
-        <v>181.24</v>
+        <v>447.14</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -589,16 +589,16 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="N2" t="n">
-        <v>4979.8</v>
+        <v>4740</v>
       </c>
       <c r="O2" t="n">
-        <v>43.12</v>
+        <v>284.4</v>
       </c>
       <c r="P2" t="n">
-        <v>0.43</v>
+        <v>2.84</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>24.47</v>
+        <v>23.31</v>
       </c>
       <c r="U2" t="n">
-        <v>15.09</v>
+        <v>30.83</v>
       </c>
       <c r="V2" t="n">
-        <v>3124.01</v>
+        <v>9398.219999999999</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -631,40 +631,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>PARKHOSPS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Refex Industries</t>
+          <t>Park Medi World</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="D3" t="n">
-        <v>24750</v>
+        <v>2320786</v>
       </c>
       <c r="E3" t="n">
-        <v>54000</v>
+        <v>6280999</v>
       </c>
       <c r="F3" t="n">
-        <v>2.18</v>
+        <v>2.71</v>
       </c>
       <c r="G3" t="n">
-        <v>179</v>
+        <v>304.1</v>
       </c>
       <c r="H3" t="n">
-        <v>208.5</v>
+        <v>391.5</v>
       </c>
       <c r="I3" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="J3" t="n">
-        <v>176.31</v>
+        <v>371.3</v>
       </c>
       <c r="K3" t="n">
-        <v>181.24</v>
+        <v>447.14</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -672,16 +672,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="N3" t="n">
-        <v>4979.8</v>
+        <v>4740</v>
       </c>
       <c r="O3" t="n">
-        <v>43.12</v>
+        <v>284.4</v>
       </c>
       <c r="P3" t="n">
-        <v>0.43</v>
+        <v>2.84</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -699,13 +699,13 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>22.71</v>
+        <v>19.46</v>
       </c>
       <c r="U3" t="n">
-        <v>11.23</v>
+        <v>35.66</v>
       </c>
       <c r="V3" t="n">
-        <v>3209.78</v>
+        <v>9910.629999999999</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -714,40 +714,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>UNIPARTS</t>
+          <t>TECHNOE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Uniparts India</t>
+          <t>Techno Elec.Engg</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="D4" t="n">
-        <v>24750</v>
+        <v>2320786</v>
       </c>
       <c r="E4" t="n">
-        <v>54000</v>
+        <v>6280999</v>
       </c>
       <c r="F4" t="n">
-        <v>2.18</v>
+        <v>2.71</v>
       </c>
       <c r="G4" t="n">
-        <v>179</v>
+        <v>304.1</v>
       </c>
       <c r="H4" t="n">
-        <v>208.5</v>
+        <v>391.5</v>
       </c>
       <c r="I4" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="J4" t="n">
-        <v>176.31</v>
+        <v>371.3</v>
       </c>
       <c r="K4" t="n">
-        <v>181.24</v>
+        <v>447.14</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="N4" t="n">
-        <v>4979.8</v>
+        <v>4740</v>
       </c>
       <c r="O4" t="n">
-        <v>43.12</v>
+        <v>284.4</v>
       </c>
       <c r="P4" t="n">
-        <v>0.43</v>
+        <v>2.84</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>21.59</v>
+        <v>15.16</v>
       </c>
       <c r="U4" t="n">
-        <v>17.6</v>
+        <v>18.66</v>
       </c>
       <c r="V4" t="n">
-        <v>3225.46</v>
+        <v>9629.620000000001</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -797,40 +797,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CMLL</t>
+          <t>ELANTAS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Caliber Mining</t>
+          <t>Elantas Beck</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="D5" t="n">
-        <v>24750</v>
+        <v>2320786</v>
       </c>
       <c r="E5" t="n">
-        <v>54000</v>
+        <v>6280999</v>
       </c>
       <c r="F5" t="n">
-        <v>2.18</v>
+        <v>2.71</v>
       </c>
       <c r="G5" t="n">
-        <v>179</v>
+        <v>304.1</v>
       </c>
       <c r="H5" t="n">
-        <v>208.5</v>
+        <v>391.5</v>
       </c>
       <c r="I5" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="J5" t="n">
-        <v>176.31</v>
+        <v>371.3</v>
       </c>
       <c r="K5" t="n">
-        <v>181.24</v>
+        <v>447.14</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -838,16 +838,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="N5" t="n">
-        <v>4979.8</v>
+        <v>4740</v>
       </c>
       <c r="O5" t="n">
-        <v>43.12</v>
+        <v>284.4</v>
       </c>
       <c r="P5" t="n">
-        <v>0.43</v>
+        <v>2.84</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -865,13 +865,13 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>21.23</v>
+        <v>21.21</v>
       </c>
       <c r="U5" t="n">
-        <v>21.59</v>
+        <v>56.86</v>
       </c>
       <c r="V5" t="n">
-        <v>3375.67</v>
+        <v>10096.98</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -880,40 +880,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SHUKRAPHAR</t>
+          <t>APTUS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shukra Pharma.</t>
+          <t>Aptus Value Hou.</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="D6" t="n">
-        <v>24750</v>
+        <v>2320786</v>
       </c>
       <c r="E6" t="n">
-        <v>54000</v>
+        <v>6280999</v>
       </c>
       <c r="F6" t="n">
-        <v>2.18</v>
+        <v>2.71</v>
       </c>
       <c r="G6" t="n">
-        <v>179</v>
+        <v>304.1</v>
       </c>
       <c r="H6" t="n">
-        <v>208.5</v>
+        <v>391.5</v>
       </c>
       <c r="I6" t="n">
-        <v>177.85</v>
+        <v>395</v>
       </c>
       <c r="J6" t="n">
-        <v>176.31</v>
+        <v>371.3</v>
       </c>
       <c r="K6" t="n">
-        <v>181.24</v>
+        <v>447.14</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -921,16 +921,16 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="N6" t="n">
-        <v>4979.8</v>
+        <v>4740</v>
       </c>
       <c r="O6" t="n">
-        <v>43.12</v>
+        <v>284.4</v>
       </c>
       <c r="P6" t="n">
-        <v>0.43</v>
+        <v>2.84</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -948,430 +948,15 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>36.98</v>
+        <v>15.41</v>
       </c>
       <c r="U6" t="n">
-        <v>88.29000000000001</v>
+        <v>10.14</v>
       </c>
       <c r="V6" t="n">
-        <v>3181.78</v>
+        <v>9966.540000000001</v>
       </c>
       <c r="W6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CAPLIPOINT</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Caplin Point Lab</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>407</v>
-      </c>
-      <c r="D7" t="n">
-        <v>13640</v>
-      </c>
-      <c r="E7" t="n">
-        <v>20800</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="G7" t="n">
-        <v>395</v>
-      </c>
-      <c r="H7" t="n">
-        <v>490</v>
-      </c>
-      <c r="I7" t="n">
-        <v>407</v>
-      </c>
-      <c r="J7" t="n">
-        <v>389.07</v>
-      </c>
-      <c r="K7" t="n">
-        <v>446.45</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>12</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4884</v>
-      </c>
-      <c r="O7" t="n">
-        <v>215.16</v>
-      </c>
-      <c r="P7" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T7" t="n">
-        <v>24.24</v>
-      </c>
-      <c r="U7" t="n">
-        <v>26.83</v>
-      </c>
-      <c r="V7" t="n">
-        <v>17825.48</v>
-      </c>
-      <c r="W7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>HAPPYFORGE</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Happy Forgings</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>407</v>
-      </c>
-      <c r="D8" t="n">
-        <v>13640</v>
-      </c>
-      <c r="E8" t="n">
-        <v>20800</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="G8" t="n">
-        <v>395</v>
-      </c>
-      <c r="H8" t="n">
-        <v>490</v>
-      </c>
-      <c r="I8" t="n">
-        <v>407</v>
-      </c>
-      <c r="J8" t="n">
-        <v>389.07</v>
-      </c>
-      <c r="K8" t="n">
-        <v>446.45</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>12</v>
-      </c>
-      <c r="N8" t="n">
-        <v>4884</v>
-      </c>
-      <c r="O8" t="n">
-        <v>215.16</v>
-      </c>
-      <c r="P8" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T8" t="n">
-        <v>18.03</v>
-      </c>
-      <c r="U8" t="n">
-        <v>51.78</v>
-      </c>
-      <c r="V8" t="n">
-        <v>16957.77</v>
-      </c>
-      <c r="W8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>EMMVEE</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Emmvee Photovol.</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>407</v>
-      </c>
-      <c r="D9" t="n">
-        <v>13640</v>
-      </c>
-      <c r="E9" t="n">
-        <v>20800</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="G9" t="n">
-        <v>395</v>
-      </c>
-      <c r="H9" t="n">
-        <v>490</v>
-      </c>
-      <c r="I9" t="n">
-        <v>407</v>
-      </c>
-      <c r="J9" t="n">
-        <v>389.07</v>
-      </c>
-      <c r="K9" t="n">
-        <v>446.45</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
-        <v>12</v>
-      </c>
-      <c r="N9" t="n">
-        <v>4884</v>
-      </c>
-      <c r="O9" t="n">
-        <v>215.16</v>
-      </c>
-      <c r="P9" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T9" t="n">
-        <v>44.62</v>
-      </c>
-      <c r="U9" t="n">
-        <v>11.74</v>
-      </c>
-      <c r="V9" t="n">
-        <v>16754.71</v>
-      </c>
-      <c r="W9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ECLERX</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>eClerx Services</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>407</v>
-      </c>
-      <c r="D10" t="n">
-        <v>13640</v>
-      </c>
-      <c r="E10" t="n">
-        <v>20800</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="G10" t="n">
-        <v>395</v>
-      </c>
-      <c r="H10" t="n">
-        <v>490</v>
-      </c>
-      <c r="I10" t="n">
-        <v>407</v>
-      </c>
-      <c r="J10" t="n">
-        <v>389.07</v>
-      </c>
-      <c r="K10" t="n">
-        <v>446.45</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>12</v>
-      </c>
-      <c r="N10" t="n">
-        <v>4884</v>
-      </c>
-      <c r="O10" t="n">
-        <v>215.16</v>
-      </c>
-      <c r="P10" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T10" t="n">
-        <v>34.42</v>
-      </c>
-      <c r="U10" t="n">
-        <v>24.37</v>
-      </c>
-      <c r="V10" t="n">
-        <v>17747.88</v>
-      </c>
-      <c r="W10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>IGIL</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>International Gemological Instit</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>407</v>
-      </c>
-      <c r="D11" t="n">
-        <v>13640</v>
-      </c>
-      <c r="E11" t="n">
-        <v>20800</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="G11" t="n">
-        <v>395</v>
-      </c>
-      <c r="H11" t="n">
-        <v>490</v>
-      </c>
-      <c r="I11" t="n">
-        <v>407</v>
-      </c>
-      <c r="J11" t="n">
-        <v>389.07</v>
-      </c>
-      <c r="K11" t="n">
-        <v>446.45</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>12</v>
-      </c>
-      <c r="N11" t="n">
-        <v>4884</v>
-      </c>
-      <c r="O11" t="n">
-        <v>215.16</v>
-      </c>
-      <c r="P11" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T11" t="n">
-        <v>69.25</v>
-      </c>
-      <c r="U11" t="n">
-        <v>25.58</v>
-      </c>
-      <c r="V11" t="n">
-        <v>17052.95</v>
-      </c>
-      <c r="W11" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement FastAPI backend for TechnoFunda swing trading web application
</commit_message>
<xml_diff>
--- a/Final_Trade_Triggers.xlsx
+++ b/Final_Trade_Triggers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,40 +548,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TARIL</t>
+          <t>544826</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T R I L</t>
+          <t>Millworks Technologies</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>395</v>
+        <v>598.7</v>
       </c>
       <c r="D2" t="n">
-        <v>2320786</v>
+        <v>950297</v>
       </c>
       <c r="E2" t="n">
-        <v>6280999</v>
+        <v>3558703</v>
       </c>
       <c r="F2" t="n">
-        <v>2.71</v>
+        <v>3.74</v>
       </c>
       <c r="G2" t="n">
-        <v>304.1</v>
+        <v>480.8</v>
       </c>
       <c r="H2" t="n">
-        <v>391.5</v>
+        <v>597.5</v>
       </c>
       <c r="I2" t="n">
-        <v>395</v>
+        <v>598.7</v>
       </c>
       <c r="J2" t="n">
-        <v>371.3</v>
+        <v>562.78</v>
       </c>
       <c r="K2" t="n">
-        <v>447.14</v>
+        <v>677.72</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -589,16 +589,16 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N2" t="n">
-        <v>4740</v>
+        <v>4789.6</v>
       </c>
       <c r="O2" t="n">
-        <v>284.4</v>
+        <v>287.36</v>
       </c>
       <c r="P2" t="n">
-        <v>2.84</v>
+        <v>2.87</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>23.31</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="U2" t="n">
-        <v>30.83</v>
+        <v>47.77</v>
       </c>
       <c r="V2" t="n">
-        <v>9398.219999999999</v>
+        <v>1772.92</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -631,40 +631,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PARKHOSPS</t>
+          <t>544773</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Park Medi World</t>
+          <t>Merritronix</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>395</v>
+        <v>222.65</v>
       </c>
       <c r="D3" t="n">
-        <v>2320786</v>
+        <v>331513</v>
       </c>
       <c r="E3" t="n">
-        <v>6280999</v>
+        <v>1041002</v>
       </c>
       <c r="F3" t="n">
-        <v>2.71</v>
+        <v>3.14</v>
       </c>
       <c r="G3" t="n">
-        <v>304.1</v>
+        <v>219.95</v>
       </c>
       <c r="H3" t="n">
-        <v>391.5</v>
+        <v>287.9</v>
       </c>
       <c r="I3" t="n">
-        <v>395</v>
+        <v>222.65</v>
       </c>
       <c r="J3" t="n">
-        <v>371.3</v>
+        <v>216.65</v>
       </c>
       <c r="K3" t="n">
-        <v>447.14</v>
+        <v>235.85</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -672,16 +672,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="N3" t="n">
-        <v>4740</v>
+        <v>4898.3</v>
       </c>
       <c r="O3" t="n">
-        <v>284.4</v>
+        <v>132</v>
       </c>
       <c r="P3" t="n">
-        <v>2.84</v>
+        <v>1.32</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -699,13 +699,13 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>19.46</v>
+        <v>41.14</v>
       </c>
       <c r="U3" t="n">
-        <v>35.66</v>
+        <v>44.17</v>
       </c>
       <c r="V3" t="n">
-        <v>9910.629999999999</v>
+        <v>711.1900000000001</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -714,40 +714,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TECHNOE</t>
+          <t>526071</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Techno Elec.Engg</t>
+          <t>Stellant Secu.</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>395</v>
+        <v>260.06</v>
       </c>
       <c r="D4" t="n">
-        <v>2320786</v>
+        <v>169109</v>
       </c>
       <c r="E4" t="n">
-        <v>6280999</v>
+        <v>262642</v>
       </c>
       <c r="F4" t="n">
-        <v>2.71</v>
+        <v>1.55</v>
       </c>
       <c r="G4" t="n">
-        <v>304.1</v>
+        <v>220</v>
       </c>
       <c r="H4" t="n">
-        <v>391.5</v>
+        <v>252.1</v>
       </c>
       <c r="I4" t="n">
-        <v>395</v>
+        <v>260.06</v>
       </c>
       <c r="J4" t="n">
-        <v>371.3</v>
+        <v>244.46</v>
       </c>
       <c r="K4" t="n">
-        <v>447.14</v>
+        <v>294.38</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="N4" t="n">
-        <v>4740</v>
+        <v>4941.14</v>
       </c>
       <c r="O4" t="n">
-        <v>284.4</v>
+        <v>296.4</v>
       </c>
       <c r="P4" t="n">
-        <v>2.84</v>
+        <v>2.96</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>15.16</v>
+        <v>71.73</v>
       </c>
       <c r="U4" t="n">
-        <v>18.66</v>
+        <v>14.83</v>
       </c>
       <c r="V4" t="n">
-        <v>9629.620000000001</v>
+        <v>544.01</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -797,40 +797,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ELANTAS</t>
+          <t>CHANDAN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Elantas Beck</t>
+          <t>Chandan Healthca</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>395</v>
+        <v>260.06</v>
       </c>
       <c r="D5" t="n">
-        <v>2320786</v>
+        <v>169109</v>
       </c>
       <c r="E5" t="n">
-        <v>6280999</v>
+        <v>262642</v>
       </c>
       <c r="F5" t="n">
-        <v>2.71</v>
+        <v>1.55</v>
       </c>
       <c r="G5" t="n">
-        <v>304.1</v>
+        <v>220</v>
       </c>
       <c r="H5" t="n">
-        <v>391.5</v>
+        <v>252.1</v>
       </c>
       <c r="I5" t="n">
-        <v>395</v>
+        <v>260.06</v>
       </c>
       <c r="J5" t="n">
-        <v>371.3</v>
+        <v>244.46</v>
       </c>
       <c r="K5" t="n">
-        <v>447.14</v>
+        <v>294.38</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -838,16 +838,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="N5" t="n">
-        <v>4740</v>
+        <v>4941.14</v>
       </c>
       <c r="O5" t="n">
-        <v>284.4</v>
+        <v>296.4</v>
       </c>
       <c r="P5" t="n">
-        <v>2.84</v>
+        <v>2.96</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -865,13 +865,13 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>21.21</v>
+        <v>23.27</v>
       </c>
       <c r="U5" t="n">
-        <v>56.86</v>
+        <v>20.87</v>
       </c>
       <c r="V5" t="n">
-        <v>10096.98</v>
+        <v>548.21</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -880,40 +880,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>APTUS</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Aptus Value Hou.</t>
+          <t>U. Y. Fincorp</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>395</v>
+        <v>260.06</v>
       </c>
       <c r="D6" t="n">
-        <v>2320786</v>
+        <v>169109</v>
       </c>
       <c r="E6" t="n">
-        <v>6280999</v>
+        <v>262642</v>
       </c>
       <c r="F6" t="n">
-        <v>2.71</v>
+        <v>1.55</v>
       </c>
       <c r="G6" t="n">
-        <v>304.1</v>
+        <v>220</v>
       </c>
       <c r="H6" t="n">
-        <v>391.5</v>
+        <v>252.1</v>
       </c>
       <c r="I6" t="n">
-        <v>395</v>
+        <v>260.06</v>
       </c>
       <c r="J6" t="n">
-        <v>371.3</v>
+        <v>244.46</v>
       </c>
       <c r="K6" t="n">
-        <v>447.14</v>
+        <v>294.38</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -921,16 +921,16 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="N6" t="n">
-        <v>4740</v>
+        <v>4941.14</v>
       </c>
       <c r="O6" t="n">
-        <v>284.4</v>
+        <v>296.4</v>
       </c>
       <c r="P6" t="n">
-        <v>2.84</v>
+        <v>2.96</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -948,15 +948,181 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>15.41</v>
+        <v>19.88</v>
       </c>
       <c r="U6" t="n">
-        <v>10.14</v>
+        <v>8.68</v>
       </c>
       <c r="V6" t="n">
-        <v>9966.540000000001</v>
+        <v>537.54</v>
       </c>
       <c r="W6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>540652</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Captain Techno.</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="D7" t="n">
+        <v>169109</v>
+      </c>
+      <c r="E7" t="n">
+        <v>262642</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G7" t="n">
+        <v>220</v>
+      </c>
+      <c r="H7" t="n">
+        <v>252.1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="J7" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="K7" t="n">
+        <v>294.38</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>19</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4941.14</v>
+      </c>
+      <c r="O7" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>29.88</v>
+      </c>
+      <c r="U7" t="n">
+        <v>46.92</v>
+      </c>
+      <c r="V7" t="n">
+        <v>545.67</v>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>543172</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cospower Engine.</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="D8" t="n">
+        <v>169109</v>
+      </c>
+      <c r="E8" t="n">
+        <v>262642</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G8" t="n">
+        <v>220</v>
+      </c>
+      <c r="H8" t="n">
+        <v>252.1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="J8" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="K8" t="n">
+        <v>294.38</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>19</v>
+      </c>
+      <c r="N8" t="n">
+        <v>4941.14</v>
+      </c>
+      <c r="O8" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="P8" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="U8" t="n">
+        <v>42.25</v>
+      </c>
+      <c r="V8" t="n">
+        <v>550.03</v>
+      </c>
+      <c r="W8" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add frontend configuration for dynamic Supabase credential loading and update trade data files
</commit_message>
<xml_diff>
--- a/Final_Trade_Triggers.xlsx
+++ b/Final_Trade_Triggers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,40 +548,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>544826</t>
+          <t>SIRCA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Millworks Technologies</t>
+          <t>Sirca Paints</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>598.7</v>
+        <v>68.89</v>
       </c>
       <c r="D2" t="n">
-        <v>950297</v>
+        <v>1753297</v>
       </c>
       <c r="E2" t="n">
-        <v>3558703</v>
+        <v>2906597</v>
       </c>
       <c r="F2" t="n">
-        <v>3.74</v>
+        <v>1.66</v>
       </c>
       <c r="G2" t="n">
-        <v>480.8</v>
+        <v>58.8</v>
       </c>
       <c r="H2" t="n">
-        <v>597.5</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>598.7</v>
+        <v>68.89</v>
       </c>
       <c r="J2" t="n">
-        <v>562.78</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>677.72</v>
+        <v>77.98</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -589,16 +589,16 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="N2" t="n">
-        <v>4789.6</v>
+        <v>4960.08</v>
       </c>
       <c r="O2" t="n">
-        <v>287.36</v>
+        <v>297.36</v>
       </c>
       <c r="P2" t="n">
-        <v>2.87</v>
+        <v>2.97</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>80.98999999999999</v>
+        <v>20.28</v>
       </c>
       <c r="U2" t="n">
-        <v>47.77</v>
+        <v>35.06</v>
       </c>
       <c r="V2" t="n">
-        <v>1772.92</v>
+        <v>2350.96</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -631,40 +631,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>544773</t>
+          <t>CANTABIL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Merritronix</t>
+          <t>Cantabil Retail</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>222.65</v>
+        <v>68.89</v>
       </c>
       <c r="D3" t="n">
-        <v>331513</v>
+        <v>1753297</v>
       </c>
       <c r="E3" t="n">
-        <v>1041002</v>
+        <v>2906597</v>
       </c>
       <c r="F3" t="n">
-        <v>3.14</v>
+        <v>1.66</v>
       </c>
       <c r="G3" t="n">
-        <v>219.95</v>
+        <v>58.8</v>
       </c>
       <c r="H3" t="n">
-        <v>287.9</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>222.65</v>
+        <v>68.89</v>
       </c>
       <c r="J3" t="n">
-        <v>216.65</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="K3" t="n">
-        <v>235.85</v>
+        <v>77.98</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -672,16 +672,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="N3" t="n">
-        <v>4898.3</v>
+        <v>4960.08</v>
       </c>
       <c r="O3" t="n">
-        <v>132</v>
+        <v>297.36</v>
       </c>
       <c r="P3" t="n">
-        <v>1.32</v>
+        <v>2.97</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -699,13 +699,13 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>41.14</v>
+        <v>19.37</v>
       </c>
       <c r="U3" t="n">
-        <v>44.17</v>
+        <v>22.36</v>
       </c>
       <c r="V3" t="n">
-        <v>711.1900000000001</v>
+        <v>2177.89</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -714,40 +714,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>526071</t>
+          <t>VINCOFE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Stellant Secu.</t>
+          <t>Vintage Coffee</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>260.06</v>
+        <v>68.89</v>
       </c>
       <c r="D4" t="n">
-        <v>169109</v>
+        <v>1753297</v>
       </c>
       <c r="E4" t="n">
-        <v>262642</v>
+        <v>2906597</v>
       </c>
       <c r="F4" t="n">
-        <v>1.55</v>
+        <v>1.66</v>
       </c>
       <c r="G4" t="n">
-        <v>220</v>
+        <v>58.8</v>
       </c>
       <c r="H4" t="n">
-        <v>252.1</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>260.06</v>
+        <v>68.89</v>
       </c>
       <c r="J4" t="n">
-        <v>244.46</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>294.38</v>
+        <v>77.98</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="N4" t="n">
-        <v>4941.14</v>
+        <v>4960.08</v>
       </c>
       <c r="O4" t="n">
-        <v>296.4</v>
+        <v>297.36</v>
       </c>
       <c r="P4" t="n">
-        <v>2.96</v>
+        <v>2.97</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>71.73</v>
+        <v>18.18</v>
       </c>
       <c r="U4" t="n">
-        <v>14.83</v>
+        <v>28.5</v>
       </c>
       <c r="V4" t="n">
-        <v>544.01</v>
+        <v>2244.35</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -797,12 +797,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CHANDAN</t>
+          <t>NGLFINE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chandan Healthca</t>
+          <t>NGL Fine Chem</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -865,13 +865,13 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>23.27</v>
+        <v>16.69</v>
       </c>
       <c r="U5" t="n">
-        <v>20.87</v>
+        <v>32.08</v>
       </c>
       <c r="V5" t="n">
-        <v>548.21</v>
+        <v>1617.97</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -880,12 +880,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U. Y. Fincorp</t>
+          <t>RACL Geartech</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -948,181 +948,15 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>19.88</v>
+        <v>16.55</v>
       </c>
       <c r="U6" t="n">
-        <v>8.68</v>
+        <v>34.48</v>
       </c>
       <c r="V6" t="n">
-        <v>537.54</v>
+        <v>1627.23</v>
       </c>
       <c r="W6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>540652</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Captain Techno.</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>260.06</v>
-      </c>
-      <c r="D7" t="n">
-        <v>169109</v>
-      </c>
-      <c r="E7" t="n">
-        <v>262642</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="G7" t="n">
-        <v>220</v>
-      </c>
-      <c r="H7" t="n">
-        <v>252.1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>260.06</v>
-      </c>
-      <c r="J7" t="n">
-        <v>244.46</v>
-      </c>
-      <c r="K7" t="n">
-        <v>294.38</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>19</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4941.14</v>
-      </c>
-      <c r="O7" t="n">
-        <v>296.4</v>
-      </c>
-      <c r="P7" t="n">
-        <v>2.96</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T7" t="n">
-        <v>29.88</v>
-      </c>
-      <c r="U7" t="n">
-        <v>46.92</v>
-      </c>
-      <c r="V7" t="n">
-        <v>545.67</v>
-      </c>
-      <c r="W7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>543172</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Cospower Engine.</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>260.06</v>
-      </c>
-      <c r="D8" t="n">
-        <v>169109</v>
-      </c>
-      <c r="E8" t="n">
-        <v>262642</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="G8" t="n">
-        <v>220</v>
-      </c>
-      <c r="H8" t="n">
-        <v>252.1</v>
-      </c>
-      <c r="I8" t="n">
-        <v>260.06</v>
-      </c>
-      <c r="J8" t="n">
-        <v>244.46</v>
-      </c>
-      <c r="K8" t="n">
-        <v>294.38</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>1:2.2</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>19</v>
-      </c>
-      <c r="N8" t="n">
-        <v>4941.14</v>
-      </c>
-      <c r="O8" t="n">
-        <v>296.4</v>
-      </c>
-      <c r="P8" t="n">
-        <v>2.96</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>Ready for EOD Trade</t>
-        </is>
-      </c>
-      <c r="T8" t="n">
-        <v>38.38</v>
-      </c>
-      <c r="U8" t="n">
-        <v>42.25</v>
-      </c>
-      <c r="V8" t="n">
-        <v>550.03</v>
-      </c>
-      <c r="W8" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update vercel configuration and trading data spreadsheets
</commit_message>
<xml_diff>
--- a/Final_Trade_Triggers.xlsx
+++ b/Final_Trade_Triggers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,40 +548,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SIRCA</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sirca Paints</t>
+          <t>Macpower CNC</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>68.89</v>
+        <v>222.65</v>
       </c>
       <c r="D2" t="n">
-        <v>1753297</v>
+        <v>331513</v>
       </c>
       <c r="E2" t="n">
-        <v>2906597</v>
+        <v>1041002</v>
       </c>
       <c r="F2" t="n">
-        <v>1.66</v>
+        <v>3.14</v>
       </c>
       <c r="G2" t="n">
-        <v>58.8</v>
+        <v>219.95</v>
       </c>
       <c r="H2" t="n">
-        <v>73.15000000000001</v>
+        <v>287.9</v>
       </c>
       <c r="I2" t="n">
-        <v>68.89</v>
+        <v>222.65</v>
       </c>
       <c r="J2" t="n">
-        <v>64.76000000000001</v>
+        <v>216.65</v>
       </c>
       <c r="K2" t="n">
-        <v>77.98</v>
+        <v>235.85</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -589,16 +589,16 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="N2" t="n">
-        <v>4960.08</v>
+        <v>4898.3</v>
       </c>
       <c r="O2" t="n">
-        <v>297.36</v>
+        <v>132</v>
       </c>
       <c r="P2" t="n">
-        <v>2.97</v>
+        <v>1.32</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>20.28</v>
+        <v>29.11</v>
       </c>
       <c r="U2" t="n">
-        <v>35.06</v>
+        <v>45.12</v>
       </c>
       <c r="V2" t="n">
-        <v>2350.96</v>
+        <v>1939.5</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -631,40 +631,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CANTABIL</t>
+          <t>AVANA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cantabil Retail</t>
+          <t>Avana Electrosystems</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>68.89</v>
+        <v>408.55</v>
       </c>
       <c r="D3" t="n">
-        <v>1753297</v>
+        <v>68075</v>
       </c>
       <c r="E3" t="n">
-        <v>2906597</v>
+        <v>141831</v>
       </c>
       <c r="F3" t="n">
-        <v>1.66</v>
+        <v>2.08</v>
       </c>
       <c r="G3" t="n">
-        <v>58.8</v>
+        <v>339.5</v>
       </c>
       <c r="H3" t="n">
-        <v>73.15000000000001</v>
+        <v>423</v>
       </c>
       <c r="I3" t="n">
-        <v>68.89</v>
+        <v>408.55</v>
       </c>
       <c r="J3" t="n">
-        <v>64.76000000000001</v>
+        <v>384.04</v>
       </c>
       <c r="K3" t="n">
-        <v>77.98</v>
+        <v>462.47</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -672,16 +672,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="N3" t="n">
-        <v>4960.08</v>
+        <v>4902.6</v>
       </c>
       <c r="O3" t="n">
-        <v>297.36</v>
+        <v>294.12</v>
       </c>
       <c r="P3" t="n">
-        <v>2.97</v>
+        <v>2.94</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -699,13 +699,13 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>19.37</v>
+        <v>38.09</v>
       </c>
       <c r="U3" t="n">
-        <v>22.36</v>
+        <v>29.72</v>
       </c>
       <c r="V3" t="n">
-        <v>2177.89</v>
+        <v>347.72</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -714,40 +714,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VINCOFE</t>
+          <t>544460</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Vintage Coffee</t>
+          <t>Patel Chem</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>68.89</v>
+        <v>408.55</v>
       </c>
       <c r="D4" t="n">
-        <v>1753297</v>
+        <v>68075</v>
       </c>
       <c r="E4" t="n">
-        <v>2906597</v>
+        <v>141831</v>
       </c>
       <c r="F4" t="n">
-        <v>1.66</v>
+        <v>2.08</v>
       </c>
       <c r="G4" t="n">
-        <v>58.8</v>
+        <v>339.5</v>
       </c>
       <c r="H4" t="n">
-        <v>73.15000000000001</v>
+        <v>423</v>
       </c>
       <c r="I4" t="n">
-        <v>68.89</v>
+        <v>408.55</v>
       </c>
       <c r="J4" t="n">
-        <v>64.76000000000001</v>
+        <v>384.04</v>
       </c>
       <c r="K4" t="n">
-        <v>77.98</v>
+        <v>462.47</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="N4" t="n">
-        <v>4960.08</v>
+        <v>4902.6</v>
       </c>
       <c r="O4" t="n">
-        <v>297.36</v>
+        <v>294.12</v>
       </c>
       <c r="P4" t="n">
-        <v>2.97</v>
+        <v>2.94</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>18.18</v>
+        <v>21.85</v>
       </c>
       <c r="U4" t="n">
-        <v>28.5</v>
+        <v>27.74</v>
       </c>
       <c r="V4" t="n">
-        <v>2244.35</v>
+        <v>348.18</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -797,40 +797,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NGLFINE</t>
+          <t>METALIC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NGL Fine Chem</t>
+          <t>Metalic Technoforge</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>260.06</v>
+        <v>408.55</v>
       </c>
       <c r="D5" t="n">
-        <v>169109</v>
+        <v>68075</v>
       </c>
       <c r="E5" t="n">
-        <v>262642</v>
+        <v>141831</v>
       </c>
       <c r="F5" t="n">
-        <v>1.55</v>
+        <v>2.08</v>
       </c>
       <c r="G5" t="n">
-        <v>220</v>
+        <v>339.5</v>
       </c>
       <c r="H5" t="n">
-        <v>252.1</v>
+        <v>423</v>
       </c>
       <c r="I5" t="n">
-        <v>260.06</v>
+        <v>408.55</v>
       </c>
       <c r="J5" t="n">
-        <v>244.46</v>
+        <v>384.04</v>
       </c>
       <c r="K5" t="n">
-        <v>294.38</v>
+        <v>462.47</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -838,16 +838,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="N5" t="n">
-        <v>4941.14</v>
+        <v>4902.6</v>
       </c>
       <c r="O5" t="n">
-        <v>296.4</v>
+        <v>294.12</v>
       </c>
       <c r="P5" t="n">
-        <v>2.96</v>
+        <v>2.94</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -865,13 +865,13 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>16.69</v>
+        <v>36.06</v>
       </c>
       <c r="U5" t="n">
-        <v>32.08</v>
+        <v>28.42</v>
       </c>
       <c r="V5" t="n">
-        <v>1617.97</v>
+        <v>350.17</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -880,40 +880,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>GANESHIN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>RACL Geartech</t>
+          <t>Ganesh Infra.</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>260.06</v>
+        <v>408.55</v>
       </c>
       <c r="D6" t="n">
-        <v>169109</v>
+        <v>68075</v>
       </c>
       <c r="E6" t="n">
-        <v>262642</v>
+        <v>141831</v>
       </c>
       <c r="F6" t="n">
-        <v>1.55</v>
+        <v>2.08</v>
       </c>
       <c r="G6" t="n">
-        <v>220</v>
+        <v>339.5</v>
       </c>
       <c r="H6" t="n">
-        <v>252.1</v>
+        <v>423</v>
       </c>
       <c r="I6" t="n">
-        <v>260.06</v>
+        <v>408.55</v>
       </c>
       <c r="J6" t="n">
-        <v>244.46</v>
+        <v>384.04</v>
       </c>
       <c r="K6" t="n">
-        <v>294.38</v>
+        <v>462.47</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -921,16 +921,16 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="N6" t="n">
-        <v>4941.14</v>
+        <v>4902.6</v>
       </c>
       <c r="O6" t="n">
-        <v>296.4</v>
+        <v>294.12</v>
       </c>
       <c r="P6" t="n">
-        <v>2.96</v>
+        <v>2.94</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -948,15 +948,98 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>16.55</v>
+        <v>18.87</v>
       </c>
       <c r="U6" t="n">
-        <v>34.48</v>
+        <v>3.67</v>
       </c>
       <c r="V6" t="n">
-        <v>1627.23</v>
+        <v>334.63</v>
       </c>
       <c r="W6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ENCOMPAS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Encompass Design</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>408.55</v>
+      </c>
+      <c r="D7" t="n">
+        <v>68075</v>
+      </c>
+      <c r="E7" t="n">
+        <v>141831</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="G7" t="n">
+        <v>339.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>423</v>
+      </c>
+      <c r="I7" t="n">
+        <v>408.55</v>
+      </c>
+      <c r="J7" t="n">
+        <v>384.04</v>
+      </c>
+      <c r="K7" t="n">
+        <v>462.47</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>12</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4902.6</v>
+      </c>
+      <c r="O7" t="n">
+        <v>294.12</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>25.62</v>
+      </c>
+      <c r="U7" t="n">
+        <v>26.04</v>
+      </c>
+      <c r="V7" t="n">
+        <v>338.99</v>
+      </c>
+      <c r="W7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update swing trading and fundamental shortlist data spreadsheets
</commit_message>
<xml_diff>
--- a/Final_Trade_Triggers.xlsx
+++ b/Final_Trade_Triggers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,40 +548,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>543997</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Macpower CNC</t>
+          <t>Organic Recyclin</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>222.65</v>
+        <v>469.65</v>
       </c>
       <c r="D2" t="n">
-        <v>331513</v>
+        <v>28278</v>
       </c>
       <c r="E2" t="n">
-        <v>1041002</v>
+        <v>58408</v>
       </c>
       <c r="F2" t="n">
-        <v>3.14</v>
+        <v>2.07</v>
       </c>
       <c r="G2" t="n">
-        <v>219.95</v>
+        <v>330</v>
       </c>
       <c r="H2" t="n">
-        <v>287.9</v>
+        <v>606</v>
       </c>
       <c r="I2" t="n">
-        <v>222.65</v>
+        <v>469.65</v>
       </c>
       <c r="J2" t="n">
-        <v>216.65</v>
+        <v>441.47</v>
       </c>
       <c r="K2" t="n">
-        <v>235.85</v>
+        <v>531.65</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -589,16 +589,16 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="N2" t="n">
-        <v>4898.3</v>
+        <v>4696.5</v>
       </c>
       <c r="O2" t="n">
-        <v>132</v>
+        <v>281.8</v>
       </c>
       <c r="P2" t="n">
-        <v>1.32</v>
+        <v>2.82</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>29.11</v>
+        <v>16.59</v>
       </c>
       <c r="U2" t="n">
-        <v>45.12</v>
+        <v>11.06</v>
       </c>
       <c r="V2" t="n">
-        <v>1939.5</v>
+        <v>318.3</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -631,40 +631,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AVANA</t>
+          <t>SYSTANGO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Avana Electrosystems</t>
+          <t>Systango Tech</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>408.55</v>
+        <v>469.65</v>
       </c>
       <c r="D3" t="n">
-        <v>68075</v>
+        <v>28278</v>
       </c>
       <c r="E3" t="n">
-        <v>141831</v>
+        <v>58408</v>
       </c>
       <c r="F3" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="G3" t="n">
-        <v>339.5</v>
+        <v>330</v>
       </c>
       <c r="H3" t="n">
-        <v>423</v>
+        <v>606</v>
       </c>
       <c r="I3" t="n">
-        <v>408.55</v>
+        <v>469.65</v>
       </c>
       <c r="J3" t="n">
-        <v>384.04</v>
+        <v>441.47</v>
       </c>
       <c r="K3" t="n">
-        <v>462.47</v>
+        <v>531.65</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -672,16 +672,16 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N3" t="n">
-        <v>4902.6</v>
+        <v>4696.5</v>
       </c>
       <c r="O3" t="n">
-        <v>294.12</v>
+        <v>281.8</v>
       </c>
       <c r="P3" t="n">
-        <v>2.94</v>
+        <v>2.82</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -699,13 +699,13 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>38.09</v>
+        <v>31.85</v>
       </c>
       <c r="U3" t="n">
-        <v>29.72</v>
+        <v>10.52</v>
       </c>
       <c r="V3" t="n">
-        <v>347.72</v>
+        <v>318.45</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -714,40 +714,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>544460</t>
+          <t>FELIX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Patel Chem</t>
+          <t>Felix Industries</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>408.55</v>
+        <v>469.65</v>
       </c>
       <c r="D4" t="n">
-        <v>68075</v>
+        <v>28278</v>
       </c>
       <c r="E4" t="n">
-        <v>141831</v>
+        <v>58408</v>
       </c>
       <c r="F4" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="G4" t="n">
-        <v>339.5</v>
+        <v>330</v>
       </c>
       <c r="H4" t="n">
-        <v>423</v>
+        <v>606</v>
       </c>
       <c r="I4" t="n">
-        <v>408.55</v>
+        <v>469.65</v>
       </c>
       <c r="J4" t="n">
-        <v>384.04</v>
+        <v>441.47</v>
       </c>
       <c r="K4" t="n">
-        <v>462.47</v>
+        <v>531.65</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N4" t="n">
-        <v>4902.6</v>
+        <v>4696.5</v>
       </c>
       <c r="O4" t="n">
-        <v>294.12</v>
+        <v>281.8</v>
       </c>
       <c r="P4" t="n">
-        <v>2.94</v>
+        <v>2.82</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -782,13 +782,13 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>21.85</v>
+        <v>19.28</v>
       </c>
       <c r="U4" t="n">
-        <v>27.74</v>
+        <v>14.97</v>
       </c>
       <c r="V4" t="n">
-        <v>348.18</v>
+        <v>301.19</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -797,40 +797,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>METALIC</t>
+          <t>544669</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Metalic Technoforge</t>
+          <t>Admach Systems</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>408.55</v>
+        <v>469.65</v>
       </c>
       <c r="D5" t="n">
-        <v>68075</v>
+        <v>28278</v>
       </c>
       <c r="E5" t="n">
-        <v>141831</v>
+        <v>58408</v>
       </c>
       <c r="F5" t="n">
-        <v>2.08</v>
+        <v>2.07</v>
       </c>
       <c r="G5" t="n">
-        <v>339.5</v>
+        <v>330</v>
       </c>
       <c r="H5" t="n">
-        <v>423</v>
+        <v>606</v>
       </c>
       <c r="I5" t="n">
-        <v>408.55</v>
+        <v>469.65</v>
       </c>
       <c r="J5" t="n">
-        <v>384.04</v>
+        <v>441.47</v>
       </c>
       <c r="K5" t="n">
-        <v>462.47</v>
+        <v>531.65</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -838,16 +838,16 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N5" t="n">
-        <v>4902.6</v>
+        <v>4696.5</v>
       </c>
       <c r="O5" t="n">
-        <v>294.12</v>
+        <v>281.8</v>
       </c>
       <c r="P5" t="n">
-        <v>2.94</v>
+        <v>2.82</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -865,13 +865,13 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>36.06</v>
+        <v>25.03</v>
       </c>
       <c r="U5" t="n">
-        <v>28.42</v>
+        <v>26.04</v>
       </c>
       <c r="V5" t="n">
-        <v>350.17</v>
+        <v>314.26</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -880,40 +880,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GANESHIN</t>
+          <t>PROSTARM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ganesh Infra.</t>
+          <t>Prostarm Info</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>408.55</v>
+        <v>68.89</v>
       </c>
       <c r="D6" t="n">
-        <v>68075</v>
+        <v>1753297</v>
       </c>
       <c r="E6" t="n">
-        <v>141831</v>
+        <v>2906597</v>
       </c>
       <c r="F6" t="n">
-        <v>2.08</v>
+        <v>1.66</v>
       </c>
       <c r="G6" t="n">
-        <v>339.5</v>
+        <v>58.8</v>
       </c>
       <c r="H6" t="n">
-        <v>423</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>408.55</v>
+        <v>68.89</v>
       </c>
       <c r="J6" t="n">
-        <v>384.04</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>462.47</v>
+        <v>77.98</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -921,16 +921,16 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="N6" t="n">
-        <v>4902.6</v>
+        <v>4960.08</v>
       </c>
       <c r="O6" t="n">
-        <v>294.12</v>
+        <v>297.36</v>
       </c>
       <c r="P6" t="n">
-        <v>2.94</v>
+        <v>2.97</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -948,13 +948,13 @@
         </is>
       </c>
       <c r="T6" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="U6" t="n">
         <v>18.87</v>
       </c>
-      <c r="U6" t="n">
-        <v>3.67</v>
-      </c>
       <c r="V6" t="n">
-        <v>334.63</v>
+        <v>720.75</v>
       </c>
       <c r="W6" t="b">
         <v>1</v>
@@ -963,40 +963,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ENCOMPAS</t>
+          <t>517286</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Encompass Design</t>
+          <t>RNIT AI Solution</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>408.55</v>
+        <v>548.15</v>
       </c>
       <c r="D7" t="n">
-        <v>68075</v>
+        <v>950915</v>
       </c>
       <c r="E7" t="n">
-        <v>141831</v>
+        <v>1481319</v>
       </c>
       <c r="F7" t="n">
-        <v>2.08</v>
+        <v>1.56</v>
       </c>
       <c r="G7" t="n">
-        <v>339.5</v>
+        <v>568.7</v>
       </c>
       <c r="H7" t="n">
-        <v>423</v>
+        <v>737.9</v>
       </c>
       <c r="I7" t="n">
-        <v>408.55</v>
+        <v>548.15</v>
       </c>
       <c r="J7" t="n">
-        <v>384.04</v>
+        <v>520.74</v>
       </c>
       <c r="K7" t="n">
-        <v>462.47</v>
+        <v>608.45</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -1004,16 +1004,16 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="N7" t="n">
-        <v>4902.6</v>
+        <v>4933.35</v>
       </c>
       <c r="O7" t="n">
-        <v>294.12</v>
+        <v>246.69</v>
       </c>
       <c r="P7" t="n">
-        <v>2.94</v>
+        <v>2.47</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1031,15 +1031,596 @@
         </is>
       </c>
       <c r="T7" t="n">
-        <v>25.62</v>
+        <v>20.15</v>
       </c>
       <c r="U7" t="n">
-        <v>26.04</v>
+        <v>68.34</v>
       </c>
       <c r="V7" t="n">
-        <v>338.99</v>
+        <v>852.16</v>
       </c>
       <c r="W7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>504605</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Uni Abex Alloy</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>548.15</v>
+      </c>
+      <c r="D8" t="n">
+        <v>950915</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1481319</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G8" t="n">
+        <v>568.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>737.9</v>
+      </c>
+      <c r="I8" t="n">
+        <v>548.15</v>
+      </c>
+      <c r="J8" t="n">
+        <v>520.74</v>
+      </c>
+      <c r="K8" t="n">
+        <v>608.45</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>9</v>
+      </c>
+      <c r="N8" t="n">
+        <v>4933.35</v>
+      </c>
+      <c r="O8" t="n">
+        <v>246.69</v>
+      </c>
+      <c r="P8" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>18.81</v>
+      </c>
+      <c r="U8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="V8" t="n">
+        <v>825.11</v>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>544434</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Neetu Yoshi</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>548.15</v>
+      </c>
+      <c r="D9" t="n">
+        <v>950915</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1481319</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G9" t="n">
+        <v>568.7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>737.9</v>
+      </c>
+      <c r="I9" t="n">
+        <v>548.15</v>
+      </c>
+      <c r="J9" t="n">
+        <v>520.74</v>
+      </c>
+      <c r="K9" t="n">
+        <v>608.45</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>9</v>
+      </c>
+      <c r="N9" t="n">
+        <v>4933.35</v>
+      </c>
+      <c r="O9" t="n">
+        <v>246.69</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>31.81</v>
+      </c>
+      <c r="U9" t="n">
+        <v>32.72</v>
+      </c>
+      <c r="V9" t="n">
+        <v>818.5599999999999</v>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SVLL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Shree Vasu Logis</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>548.15</v>
+      </c>
+      <c r="D10" t="n">
+        <v>950915</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1481319</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G10" t="n">
+        <v>568.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>737.9</v>
+      </c>
+      <c r="I10" t="n">
+        <v>548.15</v>
+      </c>
+      <c r="J10" t="n">
+        <v>520.74</v>
+      </c>
+      <c r="K10" t="n">
+        <v>608.45</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>9</v>
+      </c>
+      <c r="N10" t="n">
+        <v>4933.35</v>
+      </c>
+      <c r="O10" t="n">
+        <v>246.69</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="U10" t="n">
+        <v>119.77</v>
+      </c>
+      <c r="V10" t="n">
+        <v>857.58</v>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>543378</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CWD</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="D11" t="n">
+        <v>169109</v>
+      </c>
+      <c r="E11" t="n">
+        <v>262642</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G11" t="n">
+        <v>220</v>
+      </c>
+      <c r="H11" t="n">
+        <v>252.1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="J11" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="K11" t="n">
+        <v>294.38</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>19</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4941.14</v>
+      </c>
+      <c r="O11" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="U11" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="V11" t="n">
+        <v>625.1</v>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>544626</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Exato Technologies</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="D12" t="n">
+        <v>169109</v>
+      </c>
+      <c r="E12" t="n">
+        <v>262642</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G12" t="n">
+        <v>220</v>
+      </c>
+      <c r="H12" t="n">
+        <v>252.1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="J12" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="K12" t="n">
+        <v>294.38</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>19</v>
+      </c>
+      <c r="N12" t="n">
+        <v>4941.14</v>
+      </c>
+      <c r="O12" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="P12" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>26.73</v>
+      </c>
+      <c r="U12" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="V12" t="n">
+        <v>616.5</v>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>INFLUX</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Influx Health.</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="D13" t="n">
+        <v>169109</v>
+      </c>
+      <c r="E13" t="n">
+        <v>262642</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G13" t="n">
+        <v>220</v>
+      </c>
+      <c r="H13" t="n">
+        <v>252.1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="J13" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="K13" t="n">
+        <v>294.38</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>19</v>
+      </c>
+      <c r="N13" t="n">
+        <v>4941.14</v>
+      </c>
+      <c r="O13" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="P13" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>38.36</v>
+      </c>
+      <c r="U13" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="V13" t="n">
+        <v>625.17</v>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OSELDEVICE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>OSEL Devices</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="D14" t="n">
+        <v>169109</v>
+      </c>
+      <c r="E14" t="n">
+        <v>262642</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G14" t="n">
+        <v>220</v>
+      </c>
+      <c r="H14" t="n">
+        <v>252.1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>260.06</v>
+      </c>
+      <c r="J14" t="n">
+        <v>244.46</v>
+      </c>
+      <c r="K14" t="n">
+        <v>294.38</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1:2.2</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>19</v>
+      </c>
+      <c r="N14" t="n">
+        <v>4941.14</v>
+      </c>
+      <c r="O14" t="n">
+        <v>296.4</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Ready for EOD Trade</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="U14" t="n">
+        <v>20.72</v>
+      </c>
+      <c r="V14" t="n">
+        <v>606.08</v>
+      </c>
+      <c r="W14" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>